<commit_message>
DATA: missing + Assess
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/missing/data_understanding/all/df_match_odds_miss.xlsx
+++ b/data/england/p6_deployment/missing/data_understanding/all/df_match_odds_miss.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D734"/>
+  <dimension ref="A1:D738"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10347,20 +10347,14 @@
           <t>K0JghK0c</t>
         </is>
       </c>
-      <c r="B679" t="inlineStr">
-        <is>
-          <t>8.00</t>
-        </is>
-      </c>
-      <c r="C679" t="inlineStr">
-        <is>
-          <t>5.75</t>
-        </is>
-      </c>
-      <c r="D679" t="inlineStr">
-        <is>
-          <t>1.33</t>
-        </is>
+      <c r="B679" t="n">
+        <v>8</v>
+      </c>
+      <c r="C679" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="D679" t="n">
+        <v>1.33</v>
       </c>
     </row>
     <row r="680">
@@ -10369,20 +10363,14 @@
           <t>GhdgPLWA</t>
         </is>
       </c>
-      <c r="B680" t="inlineStr">
-        <is>
-          <t>1.20</t>
-        </is>
-      </c>
-      <c r="C680" t="inlineStr">
-        <is>
-          <t>7.50</t>
-        </is>
-      </c>
-      <c r="D680" t="inlineStr">
-        <is>
-          <t>13.00</t>
-        </is>
+      <c r="B680" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C680" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="D680" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="681">
@@ -10391,20 +10379,14 @@
           <t>l6f1Na1N</t>
         </is>
       </c>
-      <c r="B681" t="inlineStr">
-        <is>
-          <t>2.20</t>
-        </is>
-      </c>
-      <c r="C681" t="inlineStr">
-        <is>
-          <t>3.50</t>
-        </is>
-      </c>
-      <c r="D681" t="inlineStr">
-        <is>
-          <t>3.10</t>
-        </is>
+      <c r="B681" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="C681" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D681" t="n">
+        <v>3.1</v>
       </c>
     </row>
     <row r="682">
@@ -10413,20 +10395,14 @@
           <t>WQcQHwPp</t>
         </is>
       </c>
-      <c r="B682" t="inlineStr">
-        <is>
-          <t>1.75</t>
-        </is>
-      </c>
-      <c r="C682" t="inlineStr">
-        <is>
-          <t>4.20</t>
-        </is>
-      </c>
-      <c r="D682" t="inlineStr">
-        <is>
-          <t>4.00</t>
-        </is>
+      <c r="B682" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="C682" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D682" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="683">
@@ -10435,20 +10411,14 @@
           <t>bXkCusHi</t>
         </is>
       </c>
-      <c r="B683" t="inlineStr">
-        <is>
-          <t>2.70</t>
-        </is>
-      </c>
-      <c r="C683" t="inlineStr">
-        <is>
-          <t>3.25</t>
-        </is>
-      </c>
-      <c r="D683" t="inlineStr">
-        <is>
-          <t>2.60</t>
-        </is>
+      <c r="B683" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="C683" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="D683" t="n">
+        <v>2.6</v>
       </c>
     </row>
     <row r="684">
@@ -10457,20 +10427,14 @@
           <t>4hy7UG8j</t>
         </is>
       </c>
-      <c r="B684" t="inlineStr">
-        <is>
-          <t>2.55</t>
-        </is>
-      </c>
-      <c r="C684" t="inlineStr">
-        <is>
-          <t>3.10</t>
-        </is>
-      </c>
-      <c r="D684" t="inlineStr">
-        <is>
-          <t>2.90</t>
-        </is>
+      <c r="B684" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="C684" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D684" t="n">
+        <v>2.9</v>
       </c>
     </row>
     <row r="685">
@@ -10479,20 +10443,14 @@
           <t>8MkyzwoT</t>
         </is>
       </c>
-      <c r="B685" t="inlineStr">
-        <is>
-          <t>4.75</t>
-        </is>
-      </c>
-      <c r="C685" t="inlineStr">
-        <is>
-          <t>4.10</t>
-        </is>
-      </c>
-      <c r="D685" t="inlineStr">
-        <is>
-          <t>1.67</t>
-        </is>
+      <c r="B685" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="C685" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="D685" t="n">
+        <v>1.67</v>
       </c>
     </row>
     <row r="686">
@@ -10501,20 +10459,14 @@
           <t>0Ei9MyY2</t>
         </is>
       </c>
-      <c r="B686" t="inlineStr">
-        <is>
-          <t>3.75</t>
-        </is>
-      </c>
-      <c r="C686" t="inlineStr">
-        <is>
-          <t>3.75</t>
-        </is>
-      </c>
-      <c r="D686" t="inlineStr">
-        <is>
-          <t>1.73</t>
-        </is>
+      <c r="B686" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="C686" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D686" t="n">
+        <v>1.73</v>
       </c>
     </row>
     <row r="687">
@@ -10523,20 +10475,14 @@
           <t>rTas7Uuh</t>
         </is>
       </c>
-      <c r="B687" t="inlineStr">
-        <is>
-          <t>5.75</t>
-        </is>
-      </c>
-      <c r="C687" t="inlineStr">
-        <is>
-          <t>4.80</t>
-        </is>
-      </c>
-      <c r="D687" t="inlineStr">
-        <is>
-          <t>1.40</t>
-        </is>
+      <c r="B687" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="C687" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="D687" t="n">
+        <v>1.4</v>
       </c>
     </row>
     <row r="688">
@@ -10545,20 +10491,14 @@
           <t>UPZ7hVQb</t>
         </is>
       </c>
-      <c r="B688" t="inlineStr">
-        <is>
-          <t>1.11</t>
-        </is>
-      </c>
-      <c r="C688" t="inlineStr">
-        <is>
-          <t>8.50</t>
-        </is>
-      </c>
-      <c r="D688" t="inlineStr">
-        <is>
-          <t>15.00</t>
-        </is>
+      <c r="B688" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="C688" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D688" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="689">
@@ -10567,20 +10507,14 @@
           <t>zPRNPuie</t>
         </is>
       </c>
-      <c r="B689" t="inlineStr">
-        <is>
-          <t>1.45</t>
-        </is>
-      </c>
-      <c r="C689" t="inlineStr">
-        <is>
-          <t>4.50</t>
-        </is>
-      </c>
-      <c r="D689" t="inlineStr">
-        <is>
-          <t>5.50</t>
-        </is>
+      <c r="B689" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="C689" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D689" t="n">
+        <v>5.5</v>
       </c>
     </row>
     <row r="690">
@@ -10589,20 +10523,14 @@
           <t>MkDBaAbf</t>
         </is>
       </c>
-      <c r="B690" t="inlineStr">
-        <is>
-          <t>3.10</t>
-        </is>
-      </c>
-      <c r="C690" t="inlineStr">
-        <is>
-          <t>3.50</t>
-        </is>
-      </c>
-      <c r="D690" t="inlineStr">
-        <is>
-          <t>2.05</t>
-        </is>
+      <c r="B690" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="C690" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D690" t="n">
+        <v>2.05</v>
       </c>
     </row>
     <row r="691">
@@ -10611,20 +10539,14 @@
           <t>SlBjZEH8</t>
         </is>
       </c>
-      <c r="B691" t="inlineStr">
-        <is>
-          <t>1.62</t>
-        </is>
-      </c>
-      <c r="C691" t="inlineStr">
-        <is>
-          <t>4.20</t>
-        </is>
-      </c>
-      <c r="D691" t="inlineStr">
-        <is>
-          <t>3.90</t>
-        </is>
+      <c r="B691" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="C691" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D691" t="n">
+        <v>3.9</v>
       </c>
     </row>
     <row r="692">
@@ -10633,20 +10555,14 @@
           <t>EcoWEpWg</t>
         </is>
       </c>
-      <c r="B692" t="inlineStr">
-        <is>
-          <t>3.90</t>
-        </is>
-      </c>
-      <c r="C692" t="inlineStr">
-        <is>
-          <t>3.90</t>
-        </is>
-      </c>
-      <c r="D692" t="inlineStr">
-        <is>
-          <t>1.73</t>
-        </is>
+      <c r="B692" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="C692" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="D692" t="n">
+        <v>1.73</v>
       </c>
     </row>
     <row r="693">
@@ -10655,20 +10571,14 @@
           <t>z1qyZqU8</t>
         </is>
       </c>
-      <c r="B693" t="inlineStr">
-        <is>
-          <t>1.22</t>
-        </is>
-      </c>
-      <c r="C693" t="inlineStr">
-        <is>
-          <t>5.50</t>
-        </is>
-      </c>
-      <c r="D693" t="inlineStr">
-        <is>
-          <t>9.00</t>
-        </is>
+      <c r="B693" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="C693" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D693" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="694">
@@ -10677,20 +10587,14 @@
           <t>b3dRq1rR</t>
         </is>
       </c>
-      <c r="B694" t="inlineStr">
-        <is>
-          <t>1.33</t>
-        </is>
-      </c>
-      <c r="C694" t="inlineStr">
-        <is>
-          <t>4.75</t>
-        </is>
-      </c>
-      <c r="D694" t="inlineStr">
-        <is>
-          <t>6.50</t>
-        </is>
+      <c r="B694" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="C694" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="D694" t="n">
+        <v>6.5</v>
       </c>
     </row>
     <row r="695">
@@ -10699,20 +10603,14 @@
           <t>SKHfqRmo</t>
         </is>
       </c>
-      <c r="B695" t="inlineStr">
-        <is>
-          <t>3.20</t>
-        </is>
-      </c>
-      <c r="C695" t="inlineStr">
-        <is>
-          <t>3.40</t>
-        </is>
-      </c>
-      <c r="D695" t="inlineStr">
-        <is>
-          <t>2.00</t>
-        </is>
+      <c r="B695" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="C695" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D695" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="696">
@@ -10721,20 +10619,14 @@
           <t>GMD4OFmp</t>
         </is>
       </c>
-      <c r="B696" t="inlineStr">
-        <is>
-          <t>2.55</t>
-        </is>
-      </c>
-      <c r="C696" t="inlineStr">
-        <is>
-          <t>3.50</t>
-        </is>
-      </c>
-      <c r="D696" t="inlineStr">
-        <is>
-          <t>2.30</t>
-        </is>
+      <c r="B696" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="C696" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D696" t="n">
+        <v>2.3</v>
       </c>
     </row>
     <row r="697">
@@ -10743,20 +10635,14 @@
           <t>Gpl1M6p3</t>
         </is>
       </c>
-      <c r="B697" t="inlineStr">
-        <is>
-          <t>1.65</t>
-        </is>
-      </c>
-      <c r="C697" t="inlineStr">
-        <is>
-          <t>3.70</t>
-        </is>
-      </c>
-      <c r="D697" t="inlineStr">
-        <is>
-          <t>4.20</t>
-        </is>
+      <c r="B697" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="C697" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="D697" t="n">
+        <v>4.2</v>
       </c>
     </row>
     <row r="698">
@@ -10765,20 +10651,14 @@
           <t>MkTOG61s</t>
         </is>
       </c>
-      <c r="B698" t="inlineStr">
-        <is>
-          <t>5.00</t>
-        </is>
-      </c>
-      <c r="C698" t="inlineStr">
-        <is>
-          <t>4.50</t>
-        </is>
-      </c>
-      <c r="D698" t="inlineStr">
-        <is>
-          <t>1.44</t>
-        </is>
+      <c r="B698" t="n">
+        <v>5</v>
+      </c>
+      <c r="C698" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D698" t="n">
+        <v>1.44</v>
       </c>
     </row>
     <row r="699">
@@ -10787,20 +10667,14 @@
           <t>zeO4BBP1</t>
         </is>
       </c>
-      <c r="B699" t="inlineStr">
-        <is>
-          <t>3.90</t>
-        </is>
-      </c>
-      <c r="C699" t="inlineStr">
-        <is>
-          <t>4.00</t>
-        </is>
-      </c>
-      <c r="D699" t="inlineStr">
-        <is>
-          <t>1.62</t>
-        </is>
+      <c r="B699" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="C699" t="n">
+        <v>4</v>
+      </c>
+      <c r="D699" t="n">
+        <v>1.62</v>
       </c>
     </row>
     <row r="700">
@@ -10809,20 +10683,14 @@
           <t>fZscvu6l</t>
         </is>
       </c>
-      <c r="B700" t="inlineStr">
-        <is>
-          <t>3.00</t>
-        </is>
-      </c>
-      <c r="C700" t="inlineStr">
-        <is>
-          <t>3.40</t>
-        </is>
-      </c>
-      <c r="D700" t="inlineStr">
-        <is>
-          <t>2.05</t>
-        </is>
+      <c r="B700" t="n">
+        <v>3</v>
+      </c>
+      <c r="C700" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D700" t="n">
+        <v>2.05</v>
       </c>
     </row>
     <row r="701">
@@ -10831,20 +10699,14 @@
           <t>EJM6RNFa</t>
         </is>
       </c>
-      <c r="B701" t="inlineStr">
-        <is>
-          <t>2.75</t>
-        </is>
-      </c>
-      <c r="C701" t="inlineStr">
-        <is>
-          <t>4.00</t>
-        </is>
-      </c>
-      <c r="D701" t="inlineStr">
-        <is>
-          <t>2.00</t>
-        </is>
+      <c r="B701" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C701" t="n">
+        <v>4</v>
+      </c>
+      <c r="D701" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="702">
@@ -10853,20 +10715,14 @@
           <t>xIamkdK6</t>
         </is>
       </c>
-      <c r="B702" t="inlineStr">
-        <is>
-          <t>6.00</t>
-        </is>
-      </c>
-      <c r="C702" t="inlineStr">
-        <is>
-          <t>5.25</t>
-        </is>
-      </c>
-      <c r="D702" t="inlineStr">
-        <is>
-          <t>1.36</t>
-        </is>
+      <c r="B702" t="n">
+        <v>6</v>
+      </c>
+      <c r="C702" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="D702" t="n">
+        <v>1.36</v>
       </c>
     </row>
     <row r="703">
@@ -10875,20 +10731,14 @@
           <t>8veHKF2F</t>
         </is>
       </c>
-      <c r="B703" t="inlineStr">
-        <is>
-          <t>3.20</t>
-        </is>
-      </c>
-      <c r="C703" t="inlineStr">
-        <is>
-          <t>3.75</t>
-        </is>
-      </c>
-      <c r="D703" t="inlineStr">
-        <is>
-          <t>1.91</t>
-        </is>
+      <c r="B703" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="C703" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D703" t="n">
+        <v>1.91</v>
       </c>
     </row>
     <row r="704">
@@ -10897,20 +10747,14 @@
           <t>dvGWNJL7</t>
         </is>
       </c>
-      <c r="B704" t="inlineStr">
-        <is>
-          <t>1.29</t>
-        </is>
-      </c>
-      <c r="C704" t="inlineStr">
-        <is>
-          <t>5.50</t>
-        </is>
-      </c>
-      <c r="D704" t="inlineStr">
-        <is>
-          <t>6.50</t>
-        </is>
+      <c r="B704" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="C704" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D704" t="n">
+        <v>6.5</v>
       </c>
     </row>
     <row r="705">
@@ -10919,20 +10763,14 @@
           <t>rVUmmzkJ</t>
         </is>
       </c>
-      <c r="B705" t="inlineStr">
-        <is>
-          <t>3.40</t>
-        </is>
-      </c>
-      <c r="C705" t="inlineStr">
-        <is>
-          <t>3.30</t>
-        </is>
-      </c>
-      <c r="D705" t="inlineStr">
-        <is>
-          <t>1.95</t>
-        </is>
+      <c r="B705" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="C705" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D705" t="n">
+        <v>1.95</v>
       </c>
     </row>
     <row r="706">
@@ -10941,20 +10779,14 @@
           <t>rwwmB2VI</t>
         </is>
       </c>
-      <c r="B706" t="inlineStr">
-        <is>
-          <t>1.57</t>
-        </is>
-      </c>
-      <c r="C706" t="inlineStr">
-        <is>
-          <t>4.20</t>
-        </is>
-      </c>
-      <c r="D706" t="inlineStr">
-        <is>
-          <t>4.20</t>
-        </is>
+      <c r="B706" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="C706" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D706" t="n">
+        <v>4.2</v>
       </c>
     </row>
     <row r="707">
@@ -10963,20 +10795,14 @@
           <t>rD7AIOqS</t>
         </is>
       </c>
-      <c r="B707" t="inlineStr">
-        <is>
-          <t>1.50</t>
-        </is>
-      </c>
-      <c r="C707" t="inlineStr">
-        <is>
-          <t>4.33</t>
-        </is>
-      </c>
-      <c r="D707" t="inlineStr">
-        <is>
-          <t>4.75</t>
-        </is>
+      <c r="B707" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C707" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="D707" t="n">
+        <v>4.75</v>
       </c>
     </row>
     <row r="708">
@@ -10985,20 +10811,14 @@
           <t>zm42KpFF</t>
         </is>
       </c>
-      <c r="B708" t="inlineStr">
-        <is>
-          <t>3.30</t>
-        </is>
-      </c>
-      <c r="C708" t="inlineStr">
-        <is>
-          <t>3.50</t>
-        </is>
-      </c>
-      <c r="D708" t="inlineStr">
-        <is>
-          <t>1.91</t>
-        </is>
+      <c r="B708" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="C708" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D708" t="n">
+        <v>1.91</v>
       </c>
     </row>
     <row r="709">
@@ -11007,20 +10827,14 @@
           <t>8x8WhvLs</t>
         </is>
       </c>
-      <c r="B709" t="inlineStr">
-        <is>
-          <t>1.40</t>
-        </is>
-      </c>
-      <c r="C709" t="inlineStr">
-        <is>
-          <t>4.75</t>
-        </is>
-      </c>
-      <c r="D709" t="inlineStr">
-        <is>
-          <t>5.50</t>
-        </is>
+      <c r="B709" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="C709" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="D709" t="n">
+        <v>5.5</v>
       </c>
     </row>
     <row r="710">
@@ -11029,20 +10843,14 @@
           <t>zBnkBtx2</t>
         </is>
       </c>
-      <c r="B710" t="inlineStr">
-        <is>
-          <t>2.20</t>
-        </is>
-      </c>
-      <c r="C710" t="inlineStr">
-        <is>
-          <t>3.60</t>
-        </is>
-      </c>
-      <c r="D710" t="inlineStr">
-        <is>
-          <t>2.63</t>
-        </is>
+      <c r="B710" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="C710" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="D710" t="n">
+        <v>2.63</v>
       </c>
     </row>
     <row r="711">
@@ -11051,20 +10859,14 @@
           <t>lzCCMgId</t>
         </is>
       </c>
-      <c r="B711" t="inlineStr">
-        <is>
-          <t>3.60</t>
-        </is>
-      </c>
-      <c r="C711" t="inlineStr">
-        <is>
-          <t>4.10</t>
-        </is>
-      </c>
-      <c r="D711" t="inlineStr">
-        <is>
-          <t>1.70</t>
-        </is>
+      <c r="B711" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="C711" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="D711" t="n">
+        <v>1.7</v>
       </c>
     </row>
     <row r="712">
@@ -11073,20 +10875,14 @@
           <t>441uiIkf</t>
         </is>
       </c>
-      <c r="B712" t="inlineStr">
-        <is>
-          <t>2.00</t>
-        </is>
-      </c>
-      <c r="C712" t="inlineStr">
-        <is>
-          <t>3.70</t>
-        </is>
-      </c>
-      <c r="D712" t="inlineStr">
-        <is>
-          <t>2.90</t>
-        </is>
+      <c r="B712" t="n">
+        <v>2</v>
+      </c>
+      <c r="C712" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="D712" t="n">
+        <v>2.9</v>
       </c>
     </row>
     <row r="713">
@@ -11095,20 +10891,14 @@
           <t>2y3IoNDE</t>
         </is>
       </c>
-      <c r="B713" t="inlineStr">
-        <is>
-          <t>2.50</t>
-        </is>
-      </c>
-      <c r="C713" t="inlineStr">
-        <is>
-          <t>3.40</t>
-        </is>
-      </c>
-      <c r="D713" t="inlineStr">
-        <is>
-          <t>2.40</t>
-        </is>
+      <c r="B713" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C713" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D713" t="n">
+        <v>2.4</v>
       </c>
     </row>
     <row r="714">
@@ -11117,20 +10907,14 @@
           <t>SpqsD27k</t>
         </is>
       </c>
-      <c r="B714" t="inlineStr">
-        <is>
-          <t>2.38</t>
-        </is>
-      </c>
-      <c r="C714" t="inlineStr">
-        <is>
-          <t>3.30</t>
-        </is>
-      </c>
-      <c r="D714" t="inlineStr">
-        <is>
-          <t>2.60</t>
-        </is>
+      <c r="B714" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="C714" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D714" t="n">
+        <v>2.6</v>
       </c>
     </row>
     <row r="715">
@@ -11139,20 +10923,14 @@
           <t>dbvEzc5D</t>
         </is>
       </c>
-      <c r="B715" t="inlineStr">
-        <is>
-          <t>2.30</t>
-        </is>
-      </c>
-      <c r="C715" t="inlineStr">
-        <is>
-          <t>3.80</t>
-        </is>
-      </c>
-      <c r="D715" t="inlineStr">
-        <is>
-          <t>2.40</t>
-        </is>
+      <c r="B715" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="C715" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="D715" t="n">
+        <v>2.4</v>
       </c>
     </row>
     <row r="716">
@@ -11161,20 +10939,14 @@
           <t>8Aoafidn</t>
         </is>
       </c>
-      <c r="B716" t="inlineStr">
-        <is>
-          <t>4.20</t>
-        </is>
-      </c>
-      <c r="C716" t="inlineStr">
-        <is>
-          <t>4.33</t>
-        </is>
-      </c>
-      <c r="D716" t="inlineStr">
-        <is>
-          <t>1.55</t>
-        </is>
+      <c r="B716" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="C716" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="D716" t="n">
+        <v>1.55</v>
       </c>
     </row>
     <row r="717">
@@ -11183,20 +10955,14 @@
           <t>j1y6xJz1</t>
         </is>
       </c>
-      <c r="B717" t="inlineStr">
-        <is>
-          <t>1.22</t>
-        </is>
-      </c>
-      <c r="C717" t="inlineStr">
-        <is>
-          <t>5.50</t>
-        </is>
-      </c>
-      <c r="D717" t="inlineStr">
-        <is>
-          <t>9.00</t>
-        </is>
+      <c r="B717" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="C717" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D717" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="718">
@@ -11205,20 +10971,14 @@
           <t>xfH0b0cK</t>
         </is>
       </c>
-      <c r="B718" t="inlineStr">
-        <is>
-          <t>1.62</t>
-        </is>
-      </c>
-      <c r="C718" t="inlineStr">
-        <is>
-          <t>3.60</t>
-        </is>
-      </c>
-      <c r="D718" t="inlineStr">
-        <is>
-          <t>4.33</t>
-        </is>
+      <c r="B718" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="C718" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="D718" t="n">
+        <v>4.33</v>
       </c>
     </row>
     <row r="719">
@@ -11227,20 +10987,14 @@
           <t>vTUeDXfk</t>
         </is>
       </c>
-      <c r="B719" t="inlineStr">
-        <is>
-          <t>3.80</t>
-        </is>
-      </c>
-      <c r="C719" t="inlineStr">
-        <is>
-          <t>3.60</t>
-        </is>
-      </c>
-      <c r="D719" t="inlineStr">
-        <is>
-          <t>1.75</t>
-        </is>
+      <c r="B719" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="C719" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="D719" t="n">
+        <v>1.75</v>
       </c>
     </row>
     <row r="720">
@@ -11249,20 +11003,14 @@
           <t>UgqQIgXR</t>
         </is>
       </c>
-      <c r="B720" t="inlineStr">
-        <is>
-          <t>3.40</t>
-        </is>
-      </c>
-      <c r="C720" t="inlineStr">
-        <is>
-          <t>3.75</t>
-        </is>
-      </c>
-      <c r="D720" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
+      <c r="B720" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="C720" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D720" t="n">
+        <v>1.8</v>
       </c>
     </row>
     <row r="721">
@@ -11271,20 +11019,14 @@
           <t>xjwGj9eB</t>
         </is>
       </c>
-      <c r="B721" t="inlineStr">
-        <is>
-          <t>2.15</t>
-        </is>
-      </c>
-      <c r="C721" t="inlineStr">
-        <is>
-          <t>3.90</t>
-        </is>
-      </c>
-      <c r="D721" t="inlineStr">
-        <is>
-          <t>2.55</t>
-        </is>
+      <c r="B721" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="C721" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="D721" t="n">
+        <v>2.55</v>
       </c>
     </row>
     <row r="722">
@@ -11293,20 +11035,14 @@
           <t>SbOFR1Mr</t>
         </is>
       </c>
-      <c r="B722" t="inlineStr">
-        <is>
-          <t>1.50</t>
-        </is>
-      </c>
-      <c r="C722" t="inlineStr">
-        <is>
-          <t>4.50</t>
-        </is>
-      </c>
-      <c r="D722" t="inlineStr">
-        <is>
-          <t>4.33</t>
-        </is>
+      <c r="B722" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C722" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D722" t="n">
+        <v>4.33</v>
       </c>
     </row>
     <row r="723">
@@ -11315,20 +11051,14 @@
           <t>8EsqXNbL</t>
         </is>
       </c>
-      <c r="B723" t="inlineStr">
-        <is>
-          <t>4.33</t>
-        </is>
-      </c>
-      <c r="C723" t="inlineStr">
-        <is>
-          <t>4.50</t>
-        </is>
-      </c>
-      <c r="D723" t="inlineStr">
-        <is>
-          <t>1.50</t>
-        </is>
+      <c r="B723" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="C723" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D723" t="n">
+        <v>1.5</v>
       </c>
     </row>
     <row r="724">
@@ -11337,20 +11067,14 @@
           <t>0GI1dCOF</t>
         </is>
       </c>
-      <c r="B724" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="C724" t="inlineStr">
-        <is>
-          <t>3.80</t>
-        </is>
-      </c>
-      <c r="D724" t="inlineStr">
-        <is>
-          <t>4.20</t>
-        </is>
+      <c r="B724" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C724" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="D724" t="n">
+        <v>4.2</v>
       </c>
     </row>
     <row r="725">
@@ -11359,20 +11083,14 @@
           <t>OUZ4iTQ8</t>
         </is>
       </c>
-      <c r="B725" t="inlineStr">
-        <is>
-          <t>1.57</t>
-        </is>
-      </c>
-      <c r="C725" t="inlineStr">
-        <is>
-          <t>4.33</t>
-        </is>
-      </c>
-      <c r="D725" t="inlineStr">
-        <is>
-          <t>5.00</t>
-        </is>
+      <c r="B725" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="C725" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="D725" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="726">
@@ -11381,20 +11099,14 @@
           <t>KdTDk7eL</t>
         </is>
       </c>
-      <c r="B726" t="inlineStr">
-        <is>
-          <t>1.57</t>
-        </is>
-      </c>
-      <c r="C726" t="inlineStr">
-        <is>
-          <t>4.20</t>
-        </is>
-      </c>
-      <c r="D726" t="inlineStr">
-        <is>
-          <t>5.00</t>
-        </is>
+      <c r="B726" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="C726" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D726" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="727">
@@ -11403,20 +11115,14 @@
           <t>juKqpoJr</t>
         </is>
       </c>
-      <c r="B727" t="inlineStr">
-        <is>
-          <t>1.91</t>
-        </is>
-      </c>
-      <c r="C727" t="inlineStr">
-        <is>
-          <t>3.50</t>
-        </is>
-      </c>
-      <c r="D727" t="inlineStr">
-        <is>
-          <t>3.90</t>
-        </is>
+      <c r="B727" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="C727" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D727" t="n">
+        <v>3.9</v>
       </c>
     </row>
     <row r="728">
@@ -11425,20 +11131,14 @@
           <t>Cf8hrPme</t>
         </is>
       </c>
-      <c r="B728" t="inlineStr">
-        <is>
-          <t>3.10</t>
-        </is>
-      </c>
-      <c r="C728" t="inlineStr">
-        <is>
-          <t>3.70</t>
-        </is>
-      </c>
-      <c r="D728" t="inlineStr">
-        <is>
-          <t>2.15</t>
-        </is>
+      <c r="B728" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="C728" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="D728" t="n">
+        <v>2.15</v>
       </c>
     </row>
     <row r="729">
@@ -11447,20 +11147,14 @@
           <t>0U3n46AE</t>
         </is>
       </c>
-      <c r="B729" t="inlineStr">
-        <is>
-          <t>4.00</t>
-        </is>
-      </c>
-      <c r="C729" t="inlineStr">
-        <is>
-          <t>4.00</t>
-        </is>
-      </c>
-      <c r="D729" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
+      <c r="B729" t="n">
+        <v>4</v>
+      </c>
+      <c r="C729" t="n">
+        <v>4</v>
+      </c>
+      <c r="D729" t="n">
+        <v>1.8</v>
       </c>
     </row>
     <row r="730">
@@ -11469,20 +11163,14 @@
           <t>hSrRdO2l</t>
         </is>
       </c>
-      <c r="B730" t="inlineStr">
-        <is>
-          <t>3.00</t>
-        </is>
-      </c>
-      <c r="C730" t="inlineStr">
-        <is>
-          <t>3.70</t>
-        </is>
-      </c>
-      <c r="D730" t="inlineStr">
-        <is>
-          <t>2.15</t>
-        </is>
+      <c r="B730" t="n">
+        <v>3</v>
+      </c>
+      <c r="C730" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="D730" t="n">
+        <v>2.15</v>
       </c>
     </row>
     <row r="731">
@@ -11491,20 +11179,14 @@
           <t>xxfAVo4k</t>
         </is>
       </c>
-      <c r="B731" t="inlineStr">
-        <is>
-          <t>1.95</t>
-        </is>
-      </c>
-      <c r="C731" t="inlineStr">
-        <is>
-          <t>3.60</t>
-        </is>
-      </c>
-      <c r="D731" t="inlineStr">
-        <is>
-          <t>3.60</t>
-        </is>
+      <c r="B731" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="C731" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="D731" t="n">
+        <v>3.6</v>
       </c>
     </row>
     <row r="732">
@@ -11513,20 +11195,14 @@
           <t>WzmJTPY1</t>
         </is>
       </c>
-      <c r="B732" t="inlineStr">
-        <is>
-          <t>2.70</t>
-        </is>
-      </c>
-      <c r="C732" t="inlineStr">
-        <is>
-          <t>3.50</t>
-        </is>
-      </c>
-      <c r="D732" t="inlineStr">
-        <is>
-          <t>2.45</t>
-        </is>
+      <c r="B732" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="C732" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D732" t="n">
+        <v>2.45</v>
       </c>
     </row>
     <row r="733">
@@ -11535,20 +11211,14 @@
           <t>Ys2f2puR</t>
         </is>
       </c>
-      <c r="B733" t="inlineStr">
-        <is>
-          <t>2.63</t>
-        </is>
-      </c>
-      <c r="C733" t="inlineStr">
-        <is>
-          <t>3.40</t>
-        </is>
-      </c>
-      <c r="D733" t="inlineStr">
-        <is>
-          <t>2.60</t>
-        </is>
+      <c r="B733" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="C733" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D733" t="n">
+        <v>2.6</v>
       </c>
     </row>
     <row r="734">
@@ -11557,19 +11227,101 @@
           <t>pMLat3I7</t>
         </is>
       </c>
-      <c r="B734" t="inlineStr">
-        <is>
-          <t>3.80</t>
-        </is>
-      </c>
-      <c r="C734" t="inlineStr">
-        <is>
-          <t>3.60</t>
-        </is>
-      </c>
-      <c r="D734" t="inlineStr">
-        <is>
-          <t>1.91</t>
+      <c r="B734" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="C734" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="D734" t="n">
+        <v>1.91</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="1" t="inlineStr">
+        <is>
+          <t>SCsTyaGG</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>2.05</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>3.90</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="1" t="inlineStr">
+        <is>
+          <t>KnvLwLo4</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>3.50</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>3.50</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="1" t="inlineStr">
+        <is>
+          <t>WlWOlmQN</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>3.75</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>4.50</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>1.62</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="1" t="inlineStr">
+        <is>
+          <t>drCAfjgS</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>2.38</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>3.70</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>2.70</t>
         </is>
       </c>
     </row>

</xml_diff>